<commit_message>
Update model with real volumes (30 moves/mo, $1,000 ticket, 2 trucks) and add family compliance checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A79FBWhDVnBNaAoxsT5kU2
</commit_message>
<xml_diff>
--- a/model/Seckler_Modelo_Financeiro.xlsx
+++ b/model/Seckler_Modelo_Financeiro.xlsx
@@ -675,17 +675,17 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PENDENTE: histórico real da Seckler. FMCSA mostra 1 caminhão/1 motorista (localmovers.com).</t>
+          <t>Renan (17/10/2026): ~30 mudanças/mês com 2 caminhões. Conservador -20%, otimista +20%.</t>
         </is>
       </c>
     </row>
@@ -701,17 +701,17 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="D5" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>1100</v>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>1300</v>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>moveBuddha Orlando: US$672-1.550 (1-2 quartos); FreightWaves: US$306-2.712. Validar com faturas.</t>
+          <t>Renan (17/10/2026): ticket médio ~US$1.000, mínimo US$450. Coerente com moveBuddha Orlando (US$672-1.550).</t>
         </is>
       </c>
     </row>

</xml_diff>